<commit_message>
Added file tracking and missing file detection in master summary
</commit_message>
<xml_diff>
--- a/reports/Master_Comparison_Report.xlsx
+++ b/reports/Master_Comparison_Report.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,25 +433,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>CB File</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>AC File</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Differences</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Missing Records</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Zero Values</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Duplicates</t>
         </is>
@@ -470,19 +480,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00022_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00022_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -499,19 +519,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00022_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00022_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
       <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -528,19 +558,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00022_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00022_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -557,19 +597,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00023_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00023_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
       <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>1</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -586,19 +636,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00023_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00023_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -615,19 +675,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00023_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00023_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -644,19 +714,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00221_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00221_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -673,19 +753,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00221_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00221_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="F9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
       <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -702,19 +792,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00221_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>AC FILE MISSING</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -731,19 +831,29 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_00221_20260614.xml</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_00221_20260614.xml</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
       <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>1</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -760,19 +870,29 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_01254_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_01254_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
       <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -789,19 +909,29 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_01254_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_01254_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
       <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -818,19 +948,29 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_01254_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_01254_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="F14" t="n">
         <v>1</v>
       </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
       <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -847,19 +987,29 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_01480_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_01480_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -876,19 +1026,29 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_01480_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_01480_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
       <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -905,19 +1065,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_01480_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_01480_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="F17" t="n">
         <v>1</v>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
       <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -934,19 +1104,29 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_05450_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_05450_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
       <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>1</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -963,19 +1143,29 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_05450_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_05450_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -992,19 +1182,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_05450_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_05450_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1021,19 +1221,29 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_06796_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_06796_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
       <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1050,19 +1260,29 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_06796_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_06796_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="F22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
       <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1079,19 +1299,29 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_06796_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_06796_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
       <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
         <v>1</v>
       </c>
-      <c r="G23" t="n">
+      <c r="I23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1108,19 +1338,29 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_07347_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_07347_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1137,19 +1377,29 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_07347_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_07347_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1166,19 +1416,29 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_07347_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_07347_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
         <v>1</v>
       </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1195,19 +1455,29 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_08107_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_08107_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="F27" t="n">
         <v>1</v>
       </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
       <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1224,19 +1494,29 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_08107_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_08107_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="F28" t="n">
         <v>1</v>
       </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
       <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1253,19 +1533,29 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_08107_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_08107_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1282,19 +1572,29 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_08154_20260524.xml</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_08154_20260524.xml</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1311,19 +1611,29 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_08154_20260531.xml</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_08154_20260531.xml</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
         <v>1</v>
       </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1340,19 +1650,29 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>PAYROLL_EXPORT_08154_20260607.xml</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PAYROLL_EXPORT_08154_20260607.xml</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="F32" t="n">
         <v>1</v>
       </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="n">
-        <v>0</v>
-      </c>
       <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>